<commit_message>
Add comments for newsformattedresult til cloudconvert - archive TAR
</commit_message>
<xml_diff>
--- a/python developer tools/icon/newformattedresult.xlsx
+++ b/python developer tools/icon/newformattedresult.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeyuxie/Documents/GitHub/Hydrangea-GitHub-Enhancer/python developer tools/icon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{65C414F5-5BF2-3846-8274-1E6FFE882D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{318C99C3-A9B1-B645-8F59-327773F37D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15940" xr2:uid="{5EA9015E-BBF5-CE41-ACBB-BA85C5EEFED4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="2687" uniqueCount="2604">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="2709" uniqueCount="2605">
   <si>
     <t>ext.</t>
   </si>
@@ -7837,6 +7837,9 @@
   </si>
   <si>
     <t>image</t>
+  </si>
+  <si>
+    <t>archive</t>
   </si>
 </sst>
 </file>
@@ -8821,6 +8824,9 @@
       <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="D8" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -8910,7 +8916,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>49</v>
       </c>
@@ -8921,7 +8927,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>52</v>
       </c>
@@ -8932,7 +8938,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>55</v>
       </c>
@@ -8943,7 +8949,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>58</v>
       </c>
@@ -8954,7 +8960,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>61</v>
       </c>
@@ -8964,8 +8970,11 @@
       <c r="C21" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>64</v>
       </c>
@@ -8976,7 +8985,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>67</v>
       </c>
@@ -8987,7 +8996,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>70</v>
       </c>
@@ -8998,7 +9007,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>73</v>
       </c>
@@ -9009,7 +9018,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -9020,7 +9029,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>79</v>
       </c>
@@ -9031,7 +9040,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>82</v>
       </c>
@@ -9042,7 +9051,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>85</v>
       </c>
@@ -9053,7 +9062,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>88</v>
       </c>
@@ -9064,7 +9073,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>91</v>
       </c>
@@ -9075,7 +9084,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>94</v>
       </c>
@@ -9086,7 +9095,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>97</v>
       </c>
@@ -9097,7 +9106,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>100</v>
       </c>
@@ -9108,7 +9117,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>103</v>
       </c>
@@ -9119,7 +9128,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>103</v>
       </c>
@@ -9130,7 +9139,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>108</v>
       </c>
@@ -9140,8 +9149,11 @@
       <c r="C37" s="2" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D37" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>111</v>
       </c>
@@ -9152,7 +9164,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>114</v>
       </c>
@@ -9163,7 +9175,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>117</v>
       </c>
@@ -9174,7 +9186,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>120</v>
       </c>
@@ -9185,7 +9197,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>123</v>
       </c>
@@ -9196,7 +9208,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>126</v>
       </c>
@@ -9207,7 +9219,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>129</v>
       </c>
@@ -9218,7 +9230,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>132</v>
       </c>
@@ -9229,7 +9241,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>135</v>
       </c>
@@ -9240,7 +9252,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>138</v>
       </c>
@@ -9251,7 +9263,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>141</v>
       </c>
@@ -9542,6 +9554,9 @@
       <c r="C73" s="2" t="s">
         <v>217</v>
       </c>
+      <c r="D73" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
@@ -9619,6 +9634,9 @@
       <c r="C80" s="2" t="s">
         <v>237</v>
       </c>
+      <c r="D80" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
@@ -9796,7 +9814,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>285</v>
       </c>
@@ -9807,7 +9825,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>288</v>
       </c>
@@ -9818,7 +9836,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>288</v>
       </c>
@@ -9829,7 +9847,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>293</v>
       </c>
@@ -9840,7 +9858,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>296</v>
       </c>
@@ -9851,7 +9869,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>299</v>
       </c>
@@ -9862,7 +9880,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>302</v>
       </c>
@@ -9873,7 +9891,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>305</v>
       </c>
@@ -9884,7 +9902,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>308</v>
       </c>
@@ -9895,7 +9913,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>311</v>
       </c>
@@ -9906,7 +9924,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>314</v>
       </c>
@@ -9917,7 +9935,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>317</v>
       </c>
@@ -9928,7 +9946,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>320</v>
       </c>
@@ -9939,7 +9957,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>323</v>
       </c>
@@ -9950,7 +9968,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>326</v>
       </c>
@@ -9960,8 +9978,11 @@
       <c r="C111" s="2" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D111" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>329</v>
       </c>
@@ -10384,6 +10405,9 @@
       <c r="C149" s="2" t="s">
         <v>432</v>
       </c>
+      <c r="D149" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
@@ -10472,6 +10496,9 @@
       <c r="C157" s="2" t="s">
         <v>455</v>
       </c>
+      <c r="D157" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
@@ -11920,7 +11947,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
         <v>841</v>
       </c>
@@ -11931,7 +11958,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
         <v>844</v>
       </c>
@@ -11942,7 +11969,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
         <v>847</v>
       </c>
@@ -11953,7 +11980,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
         <v>850</v>
       </c>
@@ -11964,7 +11991,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" s="2" t="s">
         <v>853</v>
       </c>
@@ -11975,7 +12002,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" s="2" t="s">
         <v>856</v>
       </c>
@@ -11986,7 +12013,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
         <v>859</v>
       </c>
@@ -11996,8 +12023,11 @@
       <c r="C295" s="2" t="s">
         <v>861</v>
       </c>
-    </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D295" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
         <v>862</v>
       </c>
@@ -12008,7 +12038,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
         <v>862</v>
       </c>
@@ -12019,7 +12049,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
         <v>867</v>
       </c>
@@ -12030,7 +12060,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
         <v>870</v>
       </c>
@@ -12041,7 +12071,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
         <v>873</v>
       </c>
@@ -12052,7 +12082,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" s="2" t="s">
         <v>876</v>
       </c>
@@ -12063,7 +12093,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
         <v>879</v>
       </c>
@@ -12074,7 +12104,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
         <v>882</v>
       </c>
@@ -12085,7 +12115,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
         <v>885</v>
       </c>
@@ -12404,6 +12434,9 @@
       <c r="C331" s="2" t="s">
         <v>967</v>
       </c>
+      <c r="D331" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" s="2" t="s">
@@ -12481,6 +12514,9 @@
       <c r="C338" s="2" t="s">
         <v>988</v>
       </c>
+      <c r="D338" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
@@ -12536,6 +12572,9 @@
       <c r="C343" s="2" t="s">
         <v>1003</v>
       </c>
+      <c r="D343" s="2" t="s">
+        <v>2604</v>
+      </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
@@ -12818,7 +12857,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="369" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" s="2" t="s">
         <v>1079</v>
       </c>
@@ -12829,7 +12868,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" s="2" t="s">
         <v>1082</v>
       </c>
@@ -12840,7 +12879,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="371" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" s="2" t="s">
         <v>1085</v>
       </c>
@@ -12851,7 +12890,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" s="2" t="s">
         <v>1088</v>
       </c>
@@ -12862,7 +12901,7 @@
         <v>1090</v>
       </c>
     </row>
-    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" s="2" t="s">
         <v>1091</v>
       </c>
@@ -12873,7 +12912,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" s="2" t="s">
         <v>1091</v>
       </c>
@@ -12884,7 +12923,7 @@
         <v>1095</v>
       </c>
     </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" s="2" t="s">
         <v>1096</v>
       </c>
@@ -12895,7 +12934,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
         <v>1099</v>
       </c>
@@ -12906,7 +12945,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" s="2" t="s">
         <v>1102</v>
       </c>
@@ -12916,8 +12955,11 @@
       <c r="C377" s="2" t="s">
         <v>1104</v>
       </c>
-    </row>
-    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D377" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" s="2" t="s">
         <v>1105</v>
       </c>
@@ -12928,7 +12970,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" s="2" t="s">
         <v>1108</v>
       </c>
@@ -12939,7 +12981,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" s="2" t="s">
         <v>1111</v>
       </c>
@@ -12950,7 +12992,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" s="2" t="s">
         <v>1114</v>
       </c>
@@ -12961,7 +13003,7 @@
         <v>1116</v>
       </c>
     </row>
-    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" s="2" t="s">
         <v>1117</v>
       </c>
@@ -12972,7 +13014,7 @@
         <v>1119</v>
       </c>
     </row>
-    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" s="2" t="s">
         <v>1120</v>
       </c>
@@ -12983,7 +13025,7 @@
         <v>1122</v>
       </c>
     </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" s="2" t="s">
         <v>1123</v>
       </c>
@@ -12994,7 +13036,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" s="2" t="s">
         <v>1126</v>
       </c>
@@ -13005,7 +13047,7 @@
         <v>1128</v>
       </c>
     </row>
-    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" s="2" t="s">
         <v>1129</v>
       </c>
@@ -13016,7 +13058,7 @@
         <v>1131</v>
       </c>
     </row>
-    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" s="2" t="s">
         <v>1132</v>
       </c>
@@ -13026,8 +13068,11 @@
       <c r="C387" s="2" t="s">
         <v>1134</v>
       </c>
-    </row>
-    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D387" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" s="2" t="s">
         <v>1135</v>
       </c>
@@ -13038,7 +13083,7 @@
         <v>1137</v>
       </c>
     </row>
-    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" s="2" t="s">
         <v>1135</v>
       </c>
@@ -13049,7 +13094,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" s="2" t="s">
         <v>1135</v>
       </c>
@@ -13060,7 +13105,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" s="2" t="s">
         <v>1135</v>
       </c>
@@ -13071,7 +13116,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" s="2" t="s">
         <v>1144</v>
       </c>
@@ -13082,7 +13127,7 @@
         <v>1146</v>
       </c>
     </row>
-    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" s="2" t="s">
         <v>1147</v>
       </c>
@@ -13093,7 +13138,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" s="2" t="s">
         <v>1150</v>
       </c>
@@ -13104,7 +13149,7 @@
         <v>1152</v>
       </c>
     </row>
-    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" s="2" t="s">
         <v>1147</v>
       </c>
@@ -13115,7 +13160,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" s="2" t="s">
         <v>1155</v>
       </c>
@@ -13126,7 +13171,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="397" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" s="2" t="s">
         <v>1158</v>
       </c>
@@ -13137,7 +13182,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" s="2" t="s">
         <v>1161</v>
       </c>
@@ -13148,7 +13193,7 @@
         <v>1163</v>
       </c>
     </row>
-    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" s="2" t="s">
         <v>1164</v>
       </c>
@@ -13159,7 +13204,7 @@
         <v>1166</v>
       </c>
     </row>
-    <row r="400" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" s="2" t="s">
         <v>1167</v>
       </c>
@@ -14050,7 +14095,7 @@
         <v>1401</v>
       </c>
     </row>
-    <row r="481" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" s="2" t="s">
         <v>1402</v>
       </c>
@@ -14061,7 +14106,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="482" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" s="2" t="s">
         <v>1405</v>
       </c>
@@ -14072,7 +14117,7 @@
         <v>1407</v>
       </c>
     </row>
-    <row r="483" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" s="2" t="s">
         <v>1408</v>
       </c>
@@ -14083,7 +14128,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" s="2" t="s">
         <v>1411</v>
       </c>
@@ -14094,7 +14139,7 @@
         <v>1413</v>
       </c>
     </row>
-    <row r="485" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" s="2" t="s">
         <v>1414</v>
       </c>
@@ -14105,7 +14150,7 @@
         <v>1416</v>
       </c>
     </row>
-    <row r="486" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" s="2" t="s">
         <v>1417</v>
       </c>
@@ -14116,7 +14161,7 @@
         <v>1419</v>
       </c>
     </row>
-    <row r="487" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" s="2" t="s">
         <v>1417</v>
       </c>
@@ -14127,7 +14172,7 @@
         <v>1421</v>
       </c>
     </row>
-    <row r="488" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A488" s="2" t="s">
         <v>1417</v>
       </c>
@@ -14138,7 +14183,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="489" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" s="2" t="s">
         <v>1424</v>
       </c>
@@ -14149,7 +14194,7 @@
         <v>1426</v>
       </c>
     </row>
-    <row r="490" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" s="2" t="s">
         <v>1427</v>
       </c>
@@ -14160,7 +14205,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="491" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" s="2" t="s">
         <v>1430</v>
       </c>
@@ -14171,7 +14216,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="492" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A492" s="2" t="s">
         <v>1433</v>
       </c>
@@ -14182,7 +14227,7 @@
         <v>1435</v>
       </c>
     </row>
-    <row r="493" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A493" s="2" t="s">
         <v>1436</v>
       </c>
@@ -14192,8 +14237,11 @@
       <c r="C493" s="2" t="s">
         <v>1438</v>
       </c>
-    </row>
-    <row r="494" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D493" s="2" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="494" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A494" s="2" t="s">
         <v>1439</v>
       </c>
@@ -14204,7 +14252,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="495" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A495" s="2" t="s">
         <v>1442</v>
       </c>
@@ -14215,7 +14263,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="496" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A496" s="2" t="s">
         <v>1445</v>
       </c>
@@ -15637,7 +15685,7 @@
         <v>1815</v>
       </c>
     </row>
-    <row r="625" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="625" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A625" s="2" t="s">
         <v>1816</v>
       </c>
@@ -15648,7 +15696,7 @@
         <v>1818</v>
       </c>
     </row>
-    <row r="626" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="626" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A626" s="2" t="s">
         <v>1819</v>
       </c>
@@ -15659,7 +15707,7 @@
         <v>1821</v>
       </c>
     </row>
-    <row r="627" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="627" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A627" s="2" t="s">
         <v>1822</v>
       </c>
@@ -15670,7 +15718,7 @@
         <v>1824</v>
       </c>
     </row>
-    <row r="628" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="628" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A628" s="2" t="s">
         <v>1825</v>
       </c>
@@ -15681,7 +15729,7 @@
         <v>1827</v>
       </c>
     </row>
-    <row r="629" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="629" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A629" s="2" t="s">
         <v>1825</v>
       </c>
@@ -15692,7 +15740,7 @@
         <v>1829</v>
       </c>
     </row>
-    <row r="630" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="630" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A630" s="2" t="s">
         <v>1830</v>
       </c>
@@ -15703,7 +15751,7 @@
         <v>1832</v>
       </c>
     </row>
-    <row r="631" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="631" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A631" s="2" t="s">
         <v>1833</v>
       </c>
@@ -15714,7 +15762,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="632" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="632" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A632" s="2" t="s">
         <v>1836</v>
       </c>
@@ -15725,7 +15773,7 @@
         <v>1838</v>
       </c>
     </row>
-    <row r="633" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="633" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A633" s="2" t="s">
         <v>1839</v>
       </c>
@@ -15735,8 +15783,11 @@
       <c r="C633" s="2" t="s">
         <v>1841</v>
       </c>
-    </row>
-    <row r="634" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D633" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="634" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A634" s="2" t="s">
         <v>1842</v>
       </c>
@@ -15747,7 +15798,7 @@
         <v>1844</v>
       </c>
     </row>
-    <row r="635" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="635" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A635" s="2" t="s">
         <v>1845</v>
       </c>
@@ -15758,7 +15809,7 @@
         <v>1847</v>
       </c>
     </row>
-    <row r="636" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="636" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A636" s="2" t="s">
         <v>1848</v>
       </c>
@@ -15769,7 +15820,7 @@
         <v>1850</v>
       </c>
     </row>
-    <row r="637" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="637" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A637" s="2" t="s">
         <v>1851</v>
       </c>
@@ -15780,7 +15831,7 @@
         <v>1853</v>
       </c>
     </row>
-    <row r="638" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="638" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A638" s="2" t="s">
         <v>1851</v>
       </c>
@@ -15791,7 +15842,7 @@
         <v>1855</v>
       </c>
     </row>
-    <row r="639" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="639" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A639" s="2" t="s">
         <v>1856</v>
       </c>
@@ -15802,7 +15853,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="640" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="640" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A640" s="2" t="s">
         <v>1859</v>
       </c>
@@ -15813,7 +15864,7 @@
         <v>1861</v>
       </c>
     </row>
-    <row r="641" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="641" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A641" s="2" t="s">
         <v>1862</v>
       </c>
@@ -15824,7 +15875,7 @@
         <v>1864</v>
       </c>
     </row>
-    <row r="642" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="642" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A642" s="2" t="s">
         <v>1865</v>
       </c>
@@ -15835,7 +15886,7 @@
         <v>1867</v>
       </c>
     </row>
-    <row r="643" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="643" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A643" s="2" t="s">
         <v>1868</v>
       </c>
@@ -15846,7 +15897,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="644" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="644" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A644" s="2" t="s">
         <v>1871</v>
       </c>
@@ -15857,7 +15908,7 @@
         <v>1873</v>
       </c>
     </row>
-    <row r="645" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="645" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A645" s="2" t="s">
         <v>1874</v>
       </c>
@@ -15868,7 +15919,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="646" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="646" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A646" s="2" t="s">
         <v>1877</v>
       </c>
@@ -15879,7 +15930,7 @@
         <v>1879</v>
       </c>
     </row>
-    <row r="647" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="647" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A647" s="2" t="s">
         <v>1880</v>
       </c>
@@ -15890,7 +15941,7 @@
         <v>1882</v>
       </c>
     </row>
-    <row r="648" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="648" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A648" s="2" t="s">
         <v>1883</v>
       </c>
@@ -15901,7 +15952,7 @@
         <v>1885</v>
       </c>
     </row>
-    <row r="649" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="649" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A649" s="2" t="s">
         <v>1886</v>
       </c>
@@ -15911,8 +15962,11 @@
       <c r="C649" s="2" t="s">
         <v>1888</v>
       </c>
-    </row>
-    <row r="650" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D649" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="650" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A650" s="2" t="s">
         <v>1889</v>
       </c>
@@ -15923,7 +15977,7 @@
         <v>1891</v>
       </c>
     </row>
-    <row r="651" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="651" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A651" s="2" t="s">
         <v>1892</v>
       </c>
@@ -15934,7 +15988,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="652" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="652" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A652" s="2" t="s">
         <v>1895</v>
       </c>
@@ -15945,7 +15999,7 @@
         <v>1897</v>
       </c>
     </row>
-    <row r="653" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="653" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A653" s="2" t="s">
         <v>1898</v>
       </c>
@@ -15956,7 +16010,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="654" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="654" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A654" s="2" t="s">
         <v>1901</v>
       </c>
@@ -15967,7 +16021,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="655" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="655" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A655" s="2" t="s">
         <v>1904</v>
       </c>
@@ -15978,7 +16032,7 @@
         <v>1906</v>
       </c>
     </row>
-    <row r="656" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="656" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A656" s="2" t="s">
         <v>1907</v>
       </c>
@@ -16869,7 +16923,7 @@
         <v>2145</v>
       </c>
     </row>
-    <row r="737" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="737" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A737" s="2" t="s">
         <v>2146</v>
       </c>
@@ -16880,7 +16934,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="738" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="738" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A738" s="2" t="s">
         <v>2149</v>
       </c>
@@ -16891,7 +16945,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="739" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="739" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A739" s="2" t="s">
         <v>2152</v>
       </c>
@@ -16902,7 +16956,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="740" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="740" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A740" s="2" t="s">
         <v>2155</v>
       </c>
@@ -16913,7 +16967,7 @@
         <v>2157</v>
       </c>
     </row>
-    <row r="741" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="741" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A741" s="2" t="s">
         <v>2158</v>
       </c>
@@ -16924,7 +16978,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="742" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="742" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A742" s="2" t="s">
         <v>2161</v>
       </c>
@@ -16935,7 +16989,7 @@
         <v>2163</v>
       </c>
     </row>
-    <row r="743" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="743" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A743" s="2" t="s">
         <v>2164</v>
       </c>
@@ -16946,7 +17000,7 @@
         <v>2166</v>
       </c>
     </row>
-    <row r="744" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="744" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A744" s="2" t="s">
         <v>2167</v>
       </c>
@@ -16957,7 +17011,7 @@
         <v>2169</v>
       </c>
     </row>
-    <row r="745" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="745" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A745" s="2" t="s">
         <v>2170</v>
       </c>
@@ -16968,7 +17022,7 @@
         <v>2172</v>
       </c>
     </row>
-    <row r="746" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="746" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A746" s="2" t="s">
         <v>2173</v>
       </c>
@@ -16979,7 +17033,7 @@
         <v>2175</v>
       </c>
     </row>
-    <row r="747" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="747" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A747" s="2" t="s">
         <v>2176</v>
       </c>
@@ -16990,7 +17044,7 @@
         <v>2178</v>
       </c>
     </row>
-    <row r="748" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="748" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A748" s="2" t="s">
         <v>2179</v>
       </c>
@@ -17000,8 +17054,11 @@
       <c r="C748" s="2" t="s">
         <v>2181</v>
       </c>
-    </row>
-    <row r="749" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D748" s="2" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="749" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A749" s="2" t="s">
         <v>2182</v>
       </c>
@@ -17012,7 +17069,7 @@
         <v>2184</v>
       </c>
     </row>
-    <row r="750" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="750" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A750" s="2" t="s">
         <v>2185</v>
       </c>
@@ -17023,7 +17080,7 @@
         <v>2187</v>
       </c>
     </row>
-    <row r="751" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="751" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A751" s="2" t="s">
         <v>2188</v>
       </c>
@@ -17034,7 +17091,7 @@
         <v>2190</v>
       </c>
     </row>
-    <row r="752" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="752" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A752" s="2" t="s">
         <v>2191</v>
       </c>
@@ -17045,7 +17102,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="753" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="753" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A753" s="2" t="s">
         <v>2194</v>
       </c>
@@ -17056,7 +17113,7 @@
         <v>2196</v>
       </c>
     </row>
-    <row r="754" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="754" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A754" s="2" t="s">
         <v>2197</v>
       </c>
@@ -17067,7 +17124,7 @@
         <v>2199</v>
       </c>
     </row>
-    <row r="755" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="755" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A755" s="2" t="s">
         <v>2200</v>
       </c>
@@ -17078,7 +17135,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="756" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="756" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A756" s="2" t="s">
         <v>2203</v>
       </c>
@@ -17089,7 +17146,7 @@
         <v>2205</v>
       </c>
     </row>
-    <row r="757" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="757" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A757" s="2" t="s">
         <v>2206</v>
       </c>
@@ -17100,7 +17157,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="758" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="758" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A758" s="2" t="s">
         <v>2209</v>
       </c>
@@ -17111,7 +17168,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="759" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="759" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A759" s="2" t="s">
         <v>2212</v>
       </c>
@@ -17121,8 +17178,11 @@
       <c r="C759" s="2" t="s">
         <v>2214</v>
       </c>
-    </row>
-    <row r="760" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D759" s="2" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="760" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A760" s="2" t="s">
         <v>2215</v>
       </c>
@@ -17132,8 +17192,11 @@
       <c r="C760" s="2" t="s">
         <v>2217</v>
       </c>
-    </row>
-    <row r="761" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D760" s="2" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="761" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A761" s="2" t="s">
         <v>2218</v>
       </c>
@@ -17144,7 +17207,7 @@
         <v>2220</v>
       </c>
     </row>
-    <row r="762" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="762" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A762" s="2" t="s">
         <v>2221</v>
       </c>
@@ -17155,7 +17218,7 @@
         <v>2223</v>
       </c>
     </row>
-    <row r="763" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="763" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A763" s="2" t="s">
         <v>2224</v>
       </c>
@@ -17166,7 +17229,7 @@
         <v>2226</v>
       </c>
     </row>
-    <row r="764" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="764" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A764" s="2" t="s">
         <v>2227</v>
       </c>
@@ -17177,7 +17240,7 @@
         <v>2229</v>
       </c>
     </row>
-    <row r="765" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="765" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A765" s="2" t="s">
         <v>2230</v>
       </c>
@@ -17188,7 +17251,7 @@
         <v>2232</v>
       </c>
     </row>
-    <row r="766" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="766" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A766" s="2" t="s">
         <v>2230</v>
       </c>
@@ -17199,7 +17262,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="767" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="767" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A767" s="2" t="s">
         <v>2235</v>
       </c>
@@ -17210,7 +17273,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="768" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="768" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A768" s="2" t="s">
         <v>2238</v>
       </c>
@@ -18101,7 +18164,7 @@
         <v>2475</v>
       </c>
     </row>
-    <row r="849" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="849" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A849" s="2" t="s">
         <v>2476</v>
       </c>
@@ -18112,7 +18175,7 @@
         <v>2478</v>
       </c>
     </row>
-    <row r="850" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="850" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A850" s="2" t="s">
         <v>2479</v>
       </c>
@@ -18123,7 +18186,7 @@
         <v>2481</v>
       </c>
     </row>
-    <row r="851" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="851" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A851" s="2" t="s">
         <v>2482</v>
       </c>
@@ -18134,7 +18197,7 @@
         <v>2484</v>
       </c>
     </row>
-    <row r="852" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="852" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A852" s="2" t="s">
         <v>2485</v>
       </c>
@@ -18145,7 +18208,7 @@
         <v>2487</v>
       </c>
     </row>
-    <row r="853" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="853" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A853" s="2" t="s">
         <v>2488</v>
       </c>
@@ -18156,7 +18219,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="854" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="854" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A854" s="2" t="s">
         <v>2491</v>
       </c>
@@ -18167,7 +18230,7 @@
         <v>2493</v>
       </c>
     </row>
-    <row r="855" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="855" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A855" s="2" t="s">
         <v>2491</v>
       </c>
@@ -18178,7 +18241,7 @@
         <v>2495</v>
       </c>
     </row>
-    <row r="856" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="856" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A856" s="2" t="s">
         <v>2496</v>
       </c>
@@ -18189,7 +18252,7 @@
         <v>2498</v>
       </c>
     </row>
-    <row r="857" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="857" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A857" s="2" t="s">
         <v>2499</v>
       </c>
@@ -18200,7 +18263,7 @@
         <v>2501</v>
       </c>
     </row>
-    <row r="858" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="858" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A858" s="2" t="s">
         <v>2499</v>
       </c>
@@ -18211,7 +18274,7 @@
         <v>2503</v>
       </c>
     </row>
-    <row r="859" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="859" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A859" s="2" t="s">
         <v>2504</v>
       </c>
@@ -18222,7 +18285,7 @@
         <v>2506</v>
       </c>
     </row>
-    <row r="860" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="860" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A860" s="2" t="s">
         <v>2507</v>
       </c>
@@ -18232,8 +18295,11 @@
       <c r="C860" s="2" t="s">
         <v>2509</v>
       </c>
-    </row>
-    <row r="861" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D860" s="2" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="861" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A861" s="2" t="s">
         <v>2510</v>
       </c>
@@ -18244,7 +18310,7 @@
         <v>2512</v>
       </c>
     </row>
-    <row r="862" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="862" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A862" s="2" t="s">
         <v>2513</v>
       </c>
@@ -18255,7 +18321,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="863" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="863" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A863" s="2" t="s">
         <v>2516</v>
       </c>
@@ -18266,7 +18332,7 @@
         <v>2518</v>
       </c>
     </row>
-    <row r="864" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="864" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A864" s="2" t="s">
         <v>2519</v>
       </c>
@@ -18277,7 +18343,7 @@
         <v>2521</v>
       </c>
     </row>
-    <row r="865" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="865" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A865" s="2" t="s">
         <v>2522</v>
       </c>
@@ -18288,7 +18354,7 @@
         <v>2524</v>
       </c>
     </row>
-    <row r="866" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="866" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A866" s="2" t="s">
         <v>2525</v>
       </c>
@@ -18299,7 +18365,7 @@
         <v>2527</v>
       </c>
     </row>
-    <row r="867" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="867" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A867" s="2" t="s">
         <v>2528</v>
       </c>
@@ -18310,7 +18376,7 @@
         <v>2530</v>
       </c>
     </row>
-    <row r="868" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="868" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A868" s="2" t="s">
         <v>2531</v>
       </c>
@@ -18321,7 +18387,7 @@
         <v>2533</v>
       </c>
     </row>
-    <row r="869" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="869" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A869" s="2" t="s">
         <v>2534</v>
       </c>
@@ -18332,7 +18398,7 @@
         <v>2536</v>
       </c>
     </row>
-    <row r="870" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="870" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A870" s="2" t="s">
         <v>2537</v>
       </c>
@@ -18343,7 +18409,7 @@
         <v>2539</v>
       </c>
     </row>
-    <row r="871" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="871" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A871" s="2" t="s">
         <v>2540</v>
       </c>
@@ -18354,7 +18420,7 @@
         <v>2542</v>
       </c>
     </row>
-    <row r="872" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="872" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A872" s="2" t="s">
         <v>2543</v>
       </c>
@@ -18365,7 +18431,7 @@
         <v>2545</v>
       </c>
     </row>
-    <row r="873" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="873" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A873" s="2" t="s">
         <v>2546</v>
       </c>
@@ -18375,8 +18441,11 @@
       <c r="C873" s="2" t="s">
         <v>2548</v>
       </c>
-    </row>
-    <row r="874" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D873" s="2" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="874" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A874" s="2" t="s">
         <v>2549</v>
       </c>
@@ -18387,7 +18456,7 @@
         <v>2551</v>
       </c>
     </row>
-    <row r="875" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="875" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A875" s="2" t="s">
         <v>2552</v>
       </c>
@@ -18398,7 +18467,7 @@
         <v>2554</v>
       </c>
     </row>
-    <row r="876" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="876" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A876" s="2" t="s">
         <v>2555</v>
       </c>
@@ -18409,7 +18478,7 @@
         <v>2557</v>
       </c>
     </row>
-    <row r="877" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="877" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A877" s="2" t="s">
         <v>2558</v>
       </c>
@@ -18420,7 +18489,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="878" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="878" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A878" s="2" t="s">
         <v>2561</v>
       </c>
@@ -18431,7 +18500,7 @@
         <v>2563</v>
       </c>
     </row>
-    <row r="879" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="879" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A879" s="2" t="s">
         <v>2564</v>
       </c>
@@ -18442,7 +18511,7 @@
         <v>2566</v>
       </c>
     </row>
-    <row r="880" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="880" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A880" s="2" t="s">
         <v>2567</v>
       </c>

</xml_diff>